<commit_message>
Set page lang from locale path; add Winter Adventures UK/DE import list
- scripts.js: derive <html lang> from the /{country}/{language}/ prefix
  (e.g. /de/de -> de-DE, /gb/en -> en-GB) instead of hardcoding "en".
- Import URL list and reports for the gb/en and de/de variants.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-winter-adventures.report.xlsx
+++ b/tools/importer/reports/import-winter-adventures.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="46">
   <si>
     <t>_reportFile</t>
   </si>
@@ -61,6 +61,42 @@
     <t>https://wknd.site/us/en.html</t>
   </si>
   <si>
+    <t>de/de/winter-adventures.report.json</t>
+  </si>
+  <si>
+    <t>["carousel","columns","cards","hero"]</t>
+  </si>
+  <si>
+    <t>de/de/winter-adventures</t>
+  </si>
+  <si>
+    <t>winter-adventures</t>
+  </si>
+  <si>
+    <t>2026-09-24T23:07:14.460Z</t>
+  </si>
+  <si>
+    <t>Winterabenteuer</t>
+  </si>
+  <si>
+    <t>http://localhost:8765/de/de/winter-adventures.html</t>
+  </si>
+  <si>
+    <t>gb/en/winter-adventures.report.json</t>
+  </si>
+  <si>
+    <t>gb/en/winter-adventures</t>
+  </si>
+  <si>
+    <t>2026-09-24T23:07:09.430Z</t>
+  </si>
+  <si>
+    <t>Winter Adventures</t>
+  </si>
+  <si>
+    <t>http://localhost:8765/gb/en/winter-adventures.html</t>
+  </si>
+  <si>
     <t>us/en/adventures.report.json</t>
   </si>
   <si>
@@ -85,19 +121,10 @@
     <t>us/en/winter-adventures.report.json</t>
   </si>
   <si>
-    <t>["carousel","columns","cards","hero"]</t>
-  </si>
-  <si>
     <t>us/en/winter-adventures</t>
   </si>
   <si>
-    <t>winter-adventures</t>
-  </si>
-  <si>
     <t>2026-09-24T22:35:59.838Z</t>
-  </si>
-  <si>
-    <t>Winter Adventures</t>
   </si>
   <si>
     <t>http://localhost:8765/us/en/winter-adventures.html</t>
@@ -510,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
@@ -605,51 +632,103 @@
         <v>23</v>
       </c>
       <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
         <v>24</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
         <v>26</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>27</v>
-      </c>
-      <c r="G4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
         <v>30</v>
-      </c>
-      <c r="B5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" t="s">
-        <v>32</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
       </c>
       <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" t="s">
         <v>33</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>34</v>
       </c>
-      <c r="G5" t="s">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>35</v>
       </c>
-      <c r="H5" t="s">
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
         <v>36</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>